<commit_message>
Feat: web-native premium memo on Vercel + valuation-depth samples
- generate_samples: fetch sector peers and pass into the package; write the
  rendered memo as site/deals/<slug>.html (live web memo, not a PDF embed).
- ic_memo.html: @media screen layout so the memo reads as a centered premium
  'paper' in the browser, not just A4 print.
- site/index.html: hero + cards now open the live web memos (DCF, trading
  comps, football field visible); PDF/Excel kept as downloads.
- tests/test_valuation.py: 10 checks on the DCF/comps/football wiring.
- Regenerated samples on live data (Persistent DCF Rs1,471 vs Rs4,683 market
  honestly flags the multiple; one no-data peer dropped, not faked).

38/38 tests green. Vercel auto-deploys site/ on push — no manual step.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/dev/project_anchor_model.xlsx
+++ b/samples/dev/project_anchor_model.xlsx
@@ -852,7 +852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -864,6 +864,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -912,6 +913,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -938,10 +944,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>12</v>
+        <v>12.27</v>
       </c>
       <c r="G2" t="n">
-        <v>15</v>
+        <v/>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -950,7 +956,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE — verify; 46.8% from promoters + open offer</t>
+          <t>VERIFIED — Ambuja to acquire 46.8% of Orient Cement (37.9% promoters + 8.9% public) at equity value Rs 8100 cr; open offer 26% at Rs 395.40/sh = 12.27% premium to Rs 352.2 prev close; announced 22 Oct 2024; EV/EBITDA unverified</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.business-standard.com/markets/capital-market-news/ambuja-cements-to-46-8-stake-in-orient-cement-announces-open-offer-at-rs-395-40-share-124102200252_1.html</t>
         </is>
       </c>
     </row>
@@ -994,6 +1005,11 @@
           <t>ILLUSTRATIVE — verify; unlisted south-India capacity buy</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://www.bseindia.com/corporates/ann.html</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1012,7 +1028,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>7600</v>
+        <v>5379</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1020,10 +1036,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v/>
+        <v>24.1</v>
       </c>
       <c r="G4" t="n">
-        <v>11</v>
+        <v/>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1032,7 +1048,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE — verify; demerger + share swap 1:52</t>
+          <t>VERIFIED — demerger of Kesoram cement (10.75 mtpa; Sedam + Basantnagar) into UltraTech; share swap 1 UltraTech per 52 Kesoram; implied offer Rs 173.15 = 24.1% premium to Rs 139.45 prev close; deal ~Rs 5379 cr; appointed date 1 Apr 2024; scheme effective 1 Mar 2025; EV/EBITDA unverified</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://www.businesstoday.in/latest/corporate/story/ultratech-cement-to-buy-kesorams-cement-business-in-rs-5379-cr-deal-announces-swap-ratio-of-152-407773-2023-11-30</t>
         </is>
       </c>
     </row>
@@ -1076,6 +1097,11 @@
           <t>ILLUSTRATIVE — verify; distressed cement consolidation; open offer</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://www.sebi.gov.in/filings/takeovers.html</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1105,16 +1131,21 @@
         <v/>
       </c>
       <c r="G6" t="n">
-        <v>9</v>
+        <v/>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>announced</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE — verify; asset purchase; long-running closing</t>
+          <t>VERIFIED — Dec 2022 binding framework (EV Rs 5666 cr; 9.4 mtpa) fell through after JAL admitted to insolvency and JAL-UltraTech arbitration; superseded by fresh BTA 21 May 2026 with JAL (acquired by Adani under IBC) + Adani Infra at EV Rs 2850 cr for 5.2 mtpa Central region (Rewa/Churk/Chunar/Sadwa); EV/EBITDA unverified</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://www.businessupturn.com/business/dalmia-bharat-acquires-5-2-mntpa-cement-capacity-from-jal-for-rs-2850-crore</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1177,7 @@
         <v>7</v>
       </c>
       <c r="G7" t="n">
-        <v>14</v>
+        <v/>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1155,7 +1186,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE — verify; Holcim India exit incl ACC; open offers for both</t>
+          <t>VERIFIED — Holcim India exit; Adani bought 63.19% Ambuja ~Rs 385/sh; open offer 26% at Rs 385 (~7% premium; ~Rs 19880 cr); part of USD 10.5 bn Ambuja+ACC deal; EV/EBITDA unverified</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://www.adani.com/newsroom/media-releases/adani-to-acquire-holcims-stake-in-ambuja-cements-and-acc-limited</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1223,7 @@
         <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>12</v>
+        <v/>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1196,7 +1232,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>ILLUSTRATIVE — verify; acquired via Ambuja/Holcim transaction</t>
+          <t>VERIFIED — acquired via Ambuja/Holcim (Holcim held 54.53% incl 50.05% via Ambuja); open offer 26% at Rs 2300 (~7% premium; ~Rs 11260 cr); part of USD 10.5 bn deal; EV/EBITDA unverified</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://www.adani.com/newsroom/media-releases/adani-to-acquire-holcims-stake-in-ambuja-cements-and-acc-limited</t>
         </is>
       </c>
     </row>

</xml_diff>